<commit_message>
Full architecture, abalation, & statistical tests rerun. Also removed some redundant files and updated statistical test scripts.
</commit_message>
<xml_diff>
--- a/Analysis/Sensitivity_alpha_sweep_deepseek.xlsx
+++ b/Analysis/Sensitivity_alpha_sweep_deepseek.xlsx
@@ -491,19 +491,19 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.144</v>
+        <v>0.12478</v>
       </c>
       <c r="G2" t="n">
-        <v>0.14522</v>
+        <v>0.13128</v>
       </c>
       <c r="H2" t="n">
-        <v>0.36682</v>
+        <v>0.39078</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7221</v>
+        <v>0.72922</v>
       </c>
       <c r="J2" t="n">
-        <v>193.6</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.30668</v>
+        <v>0.2530015384615384</v>
       </c>
       <c r="G3" t="n">
-        <v>0.33078</v>
+        <v>0.2692251282051282</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5353800000000001</v>
+        <v>0.4830725128205128</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8112999999999999</v>
+        <v>0.8164088205128206</v>
       </c>
       <c r="J3" t="n">
         <v>195</v>
@@ -567,19 +567,19 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.89732</v>
+        <v>0.8564177435897437</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9101399999999999</v>
+        <v>0.8743598974358975</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9076000000000001</v>
+        <v>0.8861507692307693</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9774200000000001</v>
+        <v>0.9651174358974359</v>
       </c>
       <c r="J4" t="n">
-        <v>194.8</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5">
@@ -607,19 +607,19 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.12676</v>
+        <v>0.1159</v>
       </c>
       <c r="G5" t="n">
-        <v>0.12972</v>
+        <v>0.12358</v>
       </c>
       <c r="H5" t="n">
-        <v>0.35444</v>
+        <v>0.38872</v>
       </c>
       <c r="I5" t="n">
-        <v>0.7149</v>
+        <v>0.7220599999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>193.6</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6">
@@ -647,16 +647,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.3169400000000001</v>
+        <v>0.2728227692307692</v>
       </c>
       <c r="G6" t="n">
-        <v>0.34052</v>
+        <v>0.2963975384615385</v>
       </c>
       <c r="H6" t="n">
-        <v>0.54052</v>
+        <v>0.4964007179487179</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8122999999999999</v>
+        <v>0.833842358974359</v>
       </c>
       <c r="J6" t="n">
         <v>195</v>
@@ -687,19 +687,19 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.88842</v>
+        <v>0.828374153846154</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9039999999999999</v>
+        <v>0.8512674871794872</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9024599999999999</v>
+        <v>0.8472152820512819</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9815200000000001</v>
+        <v>0.9692321025641025</v>
       </c>
       <c r="J7" t="n">
-        <v>194.8</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8">
@@ -727,19 +727,19 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.14328</v>
+        <v>0.12548</v>
       </c>
       <c r="G8" t="n">
-        <v>0.14418</v>
+        <v>0.13178</v>
       </c>
       <c r="H8" t="n">
-        <v>0.36476</v>
+        <v>0.38974</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7220800000000001</v>
+        <v>0.73126</v>
       </c>
       <c r="J8" t="n">
-        <v>193.6</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9">
@@ -767,16 +767,16 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.31008</v>
+        <v>0.2550380512820513</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3333199999999999</v>
+        <v>0.2712824615384615</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5405</v>
+        <v>0.4841071794871795</v>
       </c>
       <c r="I9" t="n">
-        <v>0.8112999999999999</v>
+        <v>0.8194688205128206</v>
       </c>
       <c r="J9" t="n">
         <v>195</v>
@@ -807,19 +807,19 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.90076</v>
+        <v>0.8598306666666666</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9153</v>
+        <v>0.8769145641025642</v>
       </c>
       <c r="H10" t="n">
-        <v>0.91272</v>
+        <v>0.8861507692307693</v>
       </c>
       <c r="I10" t="n">
-        <v>0.98254</v>
+        <v>0.9702668717948718</v>
       </c>
       <c r="J10" t="n">
-        <v>194.8</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11">
@@ -847,19 +847,19 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.1419</v>
+        <v>0.12342</v>
       </c>
       <c r="G11" t="n">
-        <v>0.14366</v>
+        <v>0.12974</v>
       </c>
       <c r="H11" t="n">
-        <v>0.36472</v>
+        <v>0.38976</v>
       </c>
       <c r="I11" t="n">
-        <v>0.72106</v>
+        <v>0.7241</v>
       </c>
       <c r="J11" t="n">
-        <v>193.6</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12">
@@ -887,16 +887,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.30872</v>
+        <v>0.2543486153846154</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3322999999999999</v>
+        <v>0.270770358974359</v>
       </c>
       <c r="H12" t="n">
-        <v>0.53844</v>
+        <v>0.4861577435897436</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8112999999999999</v>
+        <v>0.8164088205128206</v>
       </c>
       <c r="J12" t="n">
         <v>195</v>
@@ -927,19 +927,19 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.90076</v>
+        <v>0.8564177435897437</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9153</v>
+        <v>0.8769145641025642</v>
       </c>
       <c r="H13" t="n">
-        <v>0.91272</v>
+        <v>0.8912802051282052</v>
       </c>
       <c r="I13" t="n">
-        <v>0.98254</v>
+        <v>0.9702668717948718</v>
       </c>
       <c r="J13" t="n">
-        <v>194.8</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14">
@@ -967,19 +967,19 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.15088</v>
+        <v>0.133</v>
       </c>
       <c r="G14" t="n">
-        <v>0.15504</v>
+        <v>0.14102</v>
       </c>
       <c r="H14" t="n">
-        <v>0.36992</v>
+        <v>0.39486</v>
       </c>
       <c r="I14" t="n">
-        <v>0.72416</v>
+        <v>0.73642</v>
       </c>
       <c r="J14" t="n">
-        <v>193.6</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15">
@@ -1007,16 +1007,16 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.30394</v>
+        <v>0.2570886153846154</v>
       </c>
       <c r="G15" t="n">
-        <v>0.32562</v>
+        <v>0.2748676923076923</v>
       </c>
       <c r="H15" t="n">
-        <v>0.53846</v>
+        <v>0.4881925128205128</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8082</v>
+        <v>0.8184688205128203</v>
       </c>
       <c r="J15" t="n">
         <v>195</v>
@@ -1047,19 +1047,19 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.89186</v>
+        <v>0.8591435897435897</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9086399999999999</v>
+        <v>0.8764092307692308</v>
       </c>
       <c r="H16" t="n">
-        <v>0.9076000000000001</v>
+        <v>0.8912802051282052</v>
       </c>
       <c r="I16" t="n">
-        <v>0.98254</v>
+        <v>0.9651174358974359</v>
       </c>
       <c r="J16" t="n">
-        <v>194.8</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>